<commit_message>
fixed multi execution engine
</commit_message>
<xml_diff>
--- a/datf_core/test/testprotocol/testprotocol.xlsx
+++ b/datf_core/test/testprotocol/testprotocol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_Workspaces\GitHub\DATF_Other\Databricks\QE_ATF\datf_core\test\testprotocol\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_Workspaces\GitHub\DATF_Other\Editions\QE_ATF\datf_core\test\testprotocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3663F1FF-76CF-4527-BEA4-C796F84C9BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE85D4EB-5569-480A-9BE5-94E5D92ACC45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protocol" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="49">
   <si>
     <t>Sno.</t>
   </si>
@@ -181,6 +181,12 @@
   </si>
   <si>
     <t>test/results/</t>
+  </si>
+  <si>
+    <t>protocol_engine</t>
+  </si>
+  <si>
+    <t>snowpark</t>
   </si>
 </sst>
 </file>
@@ -564,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" customWidth="1"/>
@@ -621,7 +627,20 @@
         <v>2</v>
       </c>
     </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{C863CEBC-ABFC-44BA-A351-454F3ABC0B86}">
+      <formula1>"pyspark,snowpark,databricks"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Removing rdd references and adding new test cases.
</commit_message>
<xml_diff>
--- a/datf_core/test/testprotocol/testprotocol.xlsx
+++ b/datf_core/test/testprotocol/testprotocol.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajat.yadav\Downloads\McKesson\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajat.yadav\Downloads\McKesson\New Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8D32B2-FA2F-4210-810B-A886B5628FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1551761C-EB4A-40C5-802E-433756A9C21A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="52">
   <si>
     <t>Sno.</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>testcase50_parquet_delta_match</t>
+  </si>
+  <si>
+    <t>testcase51_adls_adls_stage_removed</t>
   </si>
 </sst>
 </file>
@@ -284,7 +287,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
@@ -305,6 +308,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
@@ -654,7 +660,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333783BD-EC86-4502-A630-819DEFF8253B}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
@@ -1060,7 +1066,7 @@
         <v>41</v>
       </c>
       <c r="C27" s="4" t="str">
-        <f t="shared" ref="C27:C35" si="2">_xlfn.CONCAT("test/testcases/",B27,".xlsx")</f>
+        <f t="shared" ref="C27:C36" si="2">_xlfn.CONCAT("test/testcases/",B27,".xlsx")</f>
         <v>test/testcases/testcase26_names_fullname_etljob.xlsx</v>
       </c>
       <c r="D27" s="6" t="s">
@@ -1184,6 +1190,21 @@
         <v>test/testcases/testcase50_parquet_delta_match.xlsx</v>
       </c>
       <c r="D35" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="9">
+        <v>51</v>
+      </c>
+      <c r="B36" t="s">
+        <v>51</v>
+      </c>
+      <c r="C36" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>test/testcases/testcase51_adls_adls_stage_removed.xlsx</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1191,7 +1212,7 @@
   <autoFilter ref="A1:D25" xr:uid="{333783BD-EC86-4502-A630-819DEFF8253B}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D35" xr:uid="{864DC9FE-D2BF-46C6-8674-EF3F47262FBF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D36" xr:uid="{864DC9FE-D2BF-46C6-8674-EF3F47262FBF}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Adding new test case.
</commit_message>
<xml_diff>
--- a/datf_core/test/testprotocol/testprotocol.xlsx
+++ b/datf_core/test/testprotocol/testprotocol.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajat.yadav\Downloads\McKesson\New Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1551761C-EB4A-40C5-802E-433756A9C21A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D418B0-2FA3-47F5-ACCD-1E582CB88CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="53">
   <si>
     <t>Sno.</t>
   </si>
@@ -196,6 +196,9 @@
   </si>
   <si>
     <t>testcase51_adls_adls_stage_removed</t>
+  </si>
+  <si>
+    <t>testcase52_adls_adls_stage_manual</t>
   </si>
 </sst>
 </file>
@@ -660,7 +663,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333783BD-EC86-4502-A630-819DEFF8253B}">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
@@ -1066,7 +1069,7 @@
         <v>41</v>
       </c>
       <c r="C27" s="4" t="str">
-        <f t="shared" ref="C27:C36" si="2">_xlfn.CONCAT("test/testcases/",B27,".xlsx")</f>
+        <f t="shared" ref="C27:C37" si="2">_xlfn.CONCAT("test/testcases/",B27,".xlsx")</f>
         <v>test/testcases/testcase26_names_fullname_etljob.xlsx</v>
       </c>
       <c r="D27" s="6" t="s">
@@ -1194,7 +1197,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="9">
+      <c r="A36" s="8">
         <v>51</v>
       </c>
       <c r="B36" t="s">
@@ -1205,6 +1208,21 @@
         <v>test/testcases/testcase51_adls_adls_stage_removed.xlsx</v>
       </c>
       <c r="D36" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="9">
+        <v>52</v>
+      </c>
+      <c r="B37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>test/testcases/testcase52_adls_adls_stage_manual.xlsx</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1212,7 +1230,7 @@
   <autoFilter ref="A1:D25" xr:uid="{333783BD-EC86-4502-A630-819DEFF8253B}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D36" xr:uid="{864DC9FE-D2BF-46C6-8674-EF3F47262FBF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D37" xr:uid="{864DC9FE-D2BF-46C6-8674-EF3F47262FBF}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>